<commit_message>
docs: add missing 'report on nonexistent project' test scenario
</commit_message>
<xml_diff>
--- a/docs/Test Senaryolari - CTO Takip Sistemi.xlsx
+++ b/docs/Test Senaryolari - CTO Takip Sistemi.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -952,32 +952,32 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Aynı proje+hafta için ikinci rapor (oluşturma)</t>
+          <t>Olmayan projeye rapor ekleme</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Proje 1 hafta 29 mevcut</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>weekNumber=29</t>
+          <t>projectId=9999</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>POST /api/projects/1/reports</t>
+          <t>POST /api/projects/9999/reports</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>409 DUPLICATE_RESOURCE</t>
+          <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>409 döndü</t>
+          <t>404 döndü</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -997,22 +997,22 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Güncellemede hafta değiştirip çakışma</t>
+          <t>Aynı proje+hafta için ikinci rapor (oluşturma)</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Aynı projede başka hafta raporu var</t>
+          <t>Proje 1 hafta 29 mevcut</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>weekNumber = mevcut başka hafta</t>
+          <t>weekNumber=29</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>PUT /api/reports/{id}</t>
+          <t>POST /api/projects/1/reports</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -1042,17 +1042,17 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>İlerleme kademesinde sıra atlama</t>
+          <t>Güncellemede hafta değiştirip çakışma</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Rapor kademesi ANALIZ</t>
+          <t>Aynı projede başka hafta raporu var</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>progressStage=TAMAMLANDI</t>
+          <t>weekNumber = mevcut başka hafta</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1062,12 +1062,12 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>400 BUSINESS_RULE_VIOLATION</t>
+          <t>409 DUPLICATE_RESOURCE</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>400 döndü</t>
+          <t>409 döndü</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1087,17 +1087,17 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>İlerleme kademesini geriye alma</t>
+          <t>İlerleme kademesinde sıra atlama</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Rapor kademesi TEST</t>
+          <t>Rapor kademesi ANALIZ</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>progressStage=ANALIZ</t>
+          <t>progressStage=TAMAMLANDI</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1132,17 +1132,17 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Geçerli ilerleme (bir kademe ileri)</t>
+          <t>İlerleme kademesini geriye alma</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Rapor kademesi GELISTIRME</t>
+          <t>Rapor kademesi TEST</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>progressStage=TEST</t>
+          <t>progressStage=ANALIZ</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1152,12 +1152,12 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>200; yüzde 75'e güncellenir</t>
+          <t>400 BUSINESS_RULE_VIOLATION</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>200, %75</t>
+          <t>400 döndü</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1177,32 +1177,32 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Geçersiz enum/tarih ile rapor</t>
+          <t>Geçerli ilerleme (bir kademe ileri)</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rapor kademesi GELISTIRME</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>progressStage="COK_ILERI" / tarih="2026-13-99"</t>
+          <t>progressStage=TEST</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>POST /api/projects/{id}/reports</t>
+          <t>PUT /api/reports/{id}</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>400 INVALID_REQUEST</t>
+          <t>200; yüzde 75'e güncellenir</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>400 döndü</t>
+          <t>200, %75</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1222,130 +1222,130 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
+          <t>Geçersiz enum/tarih ile rapor</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>progressStage="COK_ILERI" / tarih="2026-13-99"</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>POST /api/projects/{id}/reports</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>400 INVALID_REQUEST</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>400 döndü</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>E2-TC9</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
           <t>Bozuk JSON gövdesi ile istek</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>{ bozuk</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>POST /api/projects/{id}/reports</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>400 INVALID_REQUEST</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>E3</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>İş kalemi yönetimi (WorkItem)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>E3-TC1</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Geçerli iş kalemi ekleme</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Kayıtlı rapor</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>{"title":"Analiz görüşmesi","status":"DEVAM_EDIYOR","assignee":"Ayşe"}</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>POST /api/reports/{id}/work-items</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>201 Created</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>201, iş kalemi eklendi</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr"/>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>E3-TC2</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Boş başlıkla iş kalemi ekleme</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>{"title":"","status":"PLANLANDI"}</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>POST /api/reports/{id}/work-items</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>400 VALIDATION_ERROR</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>400 döndü</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1360,12 +1360,12 @@
       <c r="B23" s="3" t="inlineStr"/>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>E3-TC3</t>
+          <t>E3-TC2</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Olmayan rapora iş kalemi ekleme</t>
+          <t>Boş başlıkla iş kalemi ekleme</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1375,22 +1375,22 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>reportId=999</t>
+          <t>{"title":"","status":"PLANLANDI"}</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>POST /api/reports/999/work-items</t>
+          <t>POST /api/reports/{id}/work-items</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>404 RESOURCE_NOT_FOUND</t>
+          <t>400 VALIDATION_ERROR</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>404 döndü</t>
+          <t>400 döndü</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1405,37 +1405,37 @@
       <c r="B24" s="3" t="inlineStr"/>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>E3-TC4</t>
+          <t>E3-TC3</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>İş kalemi güncelleme (başarılı)</t>
+          <t>Olmayan rapora iş kalemi ekleme</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Kayıtlı iş kalemi</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>{"title":"Güncellendi","status":"TAMAMLANDI"}</t>
+          <t>reportId=999</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>PUT /api/work-items/{id}</t>
+          <t>POST /api/reports/999/work-items</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>200; alanlar güncellenir</t>
+          <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>200, güncellendi</t>
+          <t>404 döndü</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -1450,37 +1450,37 @@
       <c r="B25" s="3" t="inlineStr"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>E3-TC5</t>
+          <t>E3-TC4</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Olmayan iş kalemi getirme/silme</t>
+          <t>İş kalemi güncelleme (başarılı)</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kayıtlı iş kalemi</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>id=9999</t>
+          <t>{"title":"Güncellendi","status":"TAMAMLANDI"}</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>GET / DELETE /api/work-items/9999</t>
+          <t>PUT /api/work-items/{id}</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>404 RESOURCE_NOT_FOUND</t>
+          <t>200; alanlar güncellenir</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>404 döndü</t>
+          <t>200, güncellendi</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1495,37 +1495,37 @@
       <c r="B26" s="3" t="inlineStr"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>E3-TC6</t>
+          <t>E3-TC5</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>İş kalemi silme (başarılı)</t>
+          <t>Olmayan iş kalemi getirme/silme</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Kayıtlı iş kalemi</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>id=9999</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>DELETE /api/work-items/{id}</t>
+          <t>GET / DELETE /api/work-items/9999</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>204 No Content</t>
+          <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>204, silindi</t>
+          <t>404 döndü</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -1540,37 +1540,37 @@
       <c r="B27" s="3" t="inlineStr"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>E3-TC7</t>
+          <t>E3-TC6</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Canlı task sayımı (DEVAM_EDIYOR)</t>
+          <t>İş kalemi silme (başarılı)</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Raporda 1 DEVAM_EDIYOR iş kalemi</t>
+          <t>Kayıtlı iş kalemi</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>id</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>GET /api/reports/{id}</t>
+          <t>DELETE /api/work-items/{id}</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>liveTaskCount = 1</t>
+          <t>204 No Content</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>liveTaskCount = 1</t>
+          <t>204, silindi</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -1578,146 +1578,146 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
-          <t>Ayrı alan tutulmaz, türetilir</t>
-        </is>
-      </c>
+      <c r="K27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr"/>
       <c r="B28" s="3" t="inlineStr"/>
       <c r="C28" s="3" t="inlineStr">
         <is>
+          <t>E3-TC7</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Canlı task sayımı (DEVAM_EDIYOR)</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Raporda 1 DEVAM_EDIYOR iş kalemi</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>GET /api/reports/{id}</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>liveTaskCount = 1</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>liveTaskCount = 1</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Ayrı alan tutulmaz, türetilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
           <t>E3-TC8</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>Rapor silinince iş kalemleri de silinir</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>Raporda iş kalemi var</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>DELETE /api/reports/{id}; sonra GET iş kalemi</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>204; iş kalemi 404 (cascade)</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>204 + 404</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K28" s="3" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>E4</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>CTO Dashboard</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>E4-TC1</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>Portföy özetini görüntüleme</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>Kayıtlı projeler</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>GET /api/dashboard/summary</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>200; tüm projeler + sayaçlar</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>200, özet döndü</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr"/>
-      <c r="B30" s="3" t="inlineStr"/>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>E4-TC2</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Risk seviyesine göre filtreleme</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>Yüksek riskli proje mevcut</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>riskLevel=YUKSEK</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>GET /api/dashboard/summary?riskLevel=YUKSEK</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>Yalnızca yüksek riskli projeler</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>Yalnızca YUKSEK döndü</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -1732,37 +1732,37 @@
       <c r="B31" s="3" t="inlineStr"/>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>E4-TC3</t>
+          <t>E4-TC2</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Raporu olmayan proje özeti</t>
+          <t>Risk seviyesine göre filtreleme</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Raporsuz proje mevcut</t>
+          <t>Yüksek riskli proje mevcut</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>riskLevel=YUKSEK</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>GET /api/dashboard/summary</t>
+          <t>GET /api/dashboard/summary?riskLevel=YUKSEK</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Proje listelenir; hasReport=false, ilerleme boş</t>
+          <t>Yalnızca yüksek riskli projeler</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>hasReport=false</t>
+          <t>Yalnızca YUKSEK döndü</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -1777,17 +1777,17 @@
       <c r="B32" s="3" t="inlineStr"/>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>E4-TC4</t>
+          <t>E4-TC3</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Boş portföy (hiç proje yok)</t>
+          <t>Raporu olmayan proje özeti</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Veritabanında proje yok</t>
+          <t>Raporsuz proje mevcut</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -1802,12 +1802,12 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>totalProjects=0; liste boş; sayaçlar 0</t>
+          <t>Proje listelenir; hasReport=false, ilerleme boş</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>0, boş liste</t>
+          <t>hasReport=false</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -1815,150 +1815,150 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t>Birim testiyle doğrulandı</t>
-        </is>
-      </c>
+      <c r="K32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr"/>
       <c r="B33" s="3" t="inlineStr"/>
       <c r="C33" s="3" t="inlineStr">
         <is>
+          <t>E4-TC4</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Boş portföy (hiç proje yok)</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Veritabanında proje yok</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>GET /api/dashboard/summary</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>totalProjects=0; liste boş; sayaçlar 0</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>0, boş liste</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Birim testiyle doğrulandı</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr"/>
+      <c r="B34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
           <t>E4-TC5</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Geçersiz risk filtresi</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>riskLevel=COK_YUKSEK</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>GET /api/dashboard/summary?riskLevel=COK_YUKSEK</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>400 INVALID_REQUEST</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr">
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
         <is>
           <t>H-3 düzeltmesi sonrası</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Genel / sistem</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>E5-TC1</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Sağlık kontrolü</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>Uygulama ayakta</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>GET /api/health</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>200; status UP, databaseStatus UP</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>200, UP</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr"/>
-      <c r="B35" s="3" t="inlineStr"/>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>E5-TC2</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>Tanımsız endpoint çağırma</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>GET /api/olmayan-endpoint</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>404 RESOURCE_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>404 döndü</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -1973,12 +1973,12 @@
       <c r="B36" s="3" t="inlineStr"/>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>E5-TC3</t>
+          <t>E5-TC2</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Desteklenmeyen HTTP metodu</t>
+          <t>Tanımsız endpoint çağırma</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -1993,17 +1993,17 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>PATCH /api/health</t>
+          <t>GET /api/olmayan-endpoint</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>405 METHOD_NOT_ALLOWED</t>
+          <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>405 döndü</t>
+          <t>404 döndü</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -2018,12 +2018,12 @@
       <c r="B37" s="3" t="inlineStr"/>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>E5-TC4</t>
+          <t>E5-TC3</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Beklenmeyen sunucu hatası</t>
+          <t>Desteklenmeyen HTTP metodu</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -2033,22 +2033,22 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>(sunucu içi beklenmeyen hata)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>İç hata tetiklenir</t>
+          <t>PATCH /api/health</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>500 INTERNAL_ERROR; teknik detay sızmaz, loglanır</t>
+          <t>405 METHOD_NOT_ALLOWED</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>500, genel mesaj</t>
+          <t>405 döndü</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -2056,56 +2056,101 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K37" s="3" t="inlineStr">
-        <is>
-          <t>Hata yönetimi testi</t>
-        </is>
-      </c>
+      <c r="K37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr"/>
       <c r="B38" s="3" t="inlineStr"/>
       <c r="C38" s="3" t="inlineStr">
         <is>
+          <t>E5-TC4</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Beklenmeyen sunucu hatası</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>(sunucu içi beklenmeyen hata)</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>İç hata tetiklenir</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>500 INTERNAL_ERROR; teknik detay sızmaz, loglanır</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>500, genel mesaj</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Hata yönetimi testi</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr"/>
+      <c r="B39" s="3" t="inlineStr"/>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
           <t>E5-TC5</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>Uygulamanın ayağa kalkması</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Uygulamayı başlat</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>Spring context sorunsuz yüklenir</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>Yüklendi</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K38" s="3" t="inlineStr">
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
         <is>
           <t>Smoke/context testi</t>
         </is>

</xml_diff>

<commit_message>
docs: split test cases into atomic scenarios and note fix->PASS history
</commit_message>
<xml_diff>
--- a/docs/Test Senaryolari - CTO Takip Sistemi.xlsx
+++ b/docs/Test Senaryolari - CTO Takip Sistemi.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>H-2 düzeltmesi sonrası</t>
+          <t>H-2: ilk testte 500 (FAIL) idi; @Size doğrulaması eklendikten sonra PASS</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>H-1 düzeltmesi sonrası</t>
+          <t>H-1: ilk testte 500 (FAIL) idi; silme öncesi rapor kontrolü eklendikten sonra PASS</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Geçersiz enum/tarih ile rapor</t>
+          <t>Tanımsız enum değeri ile rapor</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>progressStage="COK_ILERI" / tarih="2026-13-99"</t>
+          <t>progressStage="COK_ILERI"</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1267,130 +1267,130 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
+          <t>Geçersiz tarih formatı ile rapor</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>reportDate="2026-13-99"</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>POST /api/projects/{id}/reports</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>400 INVALID_REQUEST</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>400 döndü</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>E2-TC10</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
           <t>Bozuk JSON gövdesi ile istek</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>{ bozuk</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>POST /api/projects/{id}/reports</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>400 INVALID_REQUEST</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>E3</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>İş kalemi yönetimi (WorkItem)</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>E3-TC1</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Geçerli iş kalemi ekleme</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Kayıtlı rapor</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>{"title":"Analiz görüşmesi","status":"DEVAM_EDIYOR","assignee":"Ayşe"}</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>POST /api/reports/{id}/work-items</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>201 Created</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>201, iş kalemi eklendi</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr"/>
-      <c r="B23" s="3" t="inlineStr"/>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>E3-TC2</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Boş başlıkla iş kalemi ekleme</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>{"title":"","status":"PLANLANDI"}</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>POST /api/reports/{id}/work-items</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>400 VALIDATION_ERROR</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>400 döndü</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1405,12 +1405,12 @@
       <c r="B24" s="3" t="inlineStr"/>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>E3-TC3</t>
+          <t>E3-TC2</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Olmayan rapora iş kalemi ekleme</t>
+          <t>Boş başlıkla iş kalemi ekleme</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1420,22 +1420,22 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>reportId=999</t>
+          <t>{"title":"","status":"PLANLANDI"}</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>POST /api/reports/999/work-items</t>
+          <t>POST /api/reports/{id}/work-items</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>404 RESOURCE_NOT_FOUND</t>
+          <t>400 VALIDATION_ERROR</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>404 döndü</t>
+          <t>400 döndü</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -1450,37 +1450,37 @@
       <c r="B25" s="3" t="inlineStr"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>E3-TC4</t>
+          <t>E3-TC3</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>İş kalemi güncelleme (başarılı)</t>
+          <t>Olmayan rapora iş kalemi ekleme</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Kayıtlı iş kalemi</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>{"title":"Güncellendi","status":"TAMAMLANDI"}</t>
+          <t>reportId=999</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>PUT /api/work-items/{id}</t>
+          <t>POST /api/reports/999/work-items</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>200; alanlar güncellenir</t>
+          <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>200, güncellendi</t>
+          <t>404 döndü</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1495,37 +1495,37 @@
       <c r="B26" s="3" t="inlineStr"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>E3-TC5</t>
+          <t>E3-TC4</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Olmayan iş kalemi getirme/silme</t>
+          <t>İş kalemi güncelleme (başarılı)</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Kayıtlı iş kalemi</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>id=9999</t>
+          <t>{"title":"Güncellendi","status":"TAMAMLANDI"}</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>GET / DELETE /api/work-items/9999</t>
+          <t>PUT /api/work-items/{id}</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>404 RESOURCE_NOT_FOUND</t>
+          <t>200; alanlar güncellenir</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>404 döndü</t>
+          <t>200, güncellendi</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -1540,37 +1540,37 @@
       <c r="B27" s="3" t="inlineStr"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>E3-TC6</t>
+          <t>E3-TC5</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>İş kalemi silme (başarılı)</t>
+          <t>Olmayan iş kalemini getirme</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Kayıtlı iş kalemi</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>id=9999</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>DELETE /api/work-items/{id}</t>
+          <t>GET /api/work-items/9999</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>204 No Content</t>
+          <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>204, silindi</t>
+          <t>404 döndü</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -1585,37 +1585,37 @@
       <c r="B28" s="3" t="inlineStr"/>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>E3-TC7</t>
+          <t>E3-TC6</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Canlı task sayımı (DEVAM_EDIYOR)</t>
+          <t>Olmayan iş kalemini silme</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Raporda 1 DEVAM_EDIYOR iş kalemi</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>id=9999</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>GET /api/reports/{id}</t>
+          <t>DELETE /api/work-items/9999</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>liveTaskCount = 1</t>
+          <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>liveTaskCount = 1</t>
+          <t>404 döndü</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -1623,81 +1623,69 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t>Ayrı alan tutulmaz, türetilir</t>
-        </is>
-      </c>
+      <c r="K28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr"/>
       <c r="B29" s="3" t="inlineStr"/>
       <c r="C29" s="3" t="inlineStr">
         <is>
+          <t>E3-TC7</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>İş kalemi silme (başarılı)</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Kayıtlı iş kalemi</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>DELETE /api/work-items/{id}</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>204, silindi</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
           <t>E3-TC8</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Rapor silinince iş kalemleri de silinir</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>Raporda iş kalemi var</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>DELETE /api/reports/{id}; sonra GET iş kalemi</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>204; iş kalemi 404 (cascade)</t>
-        </is>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>204 + 404</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>E4</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>CTO Dashboard</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>E4-TC1</t>
-        </is>
-      </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Portföy özetini görüntüleme</t>
+          <t>Canlı task sayımı (DEVAM_EDIYOR)</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Kayıtlı projeler</t>
+          <t>Raporda 1 DEVAM_EDIYOR iş kalemi</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1707,17 +1695,17 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>GET /api/dashboard/summary</t>
+          <t>GET /api/reports/{id}</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>200; tüm projeler + sayaçlar</t>
+          <t>liveTaskCount = 1</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>200, özet döndü</t>
+          <t>liveTaskCount = 1</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -1725,44 +1713,48 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Ayrı alan tutulmaz, türetilir</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr"/>
       <c r="B31" s="3" t="inlineStr"/>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>E4-TC2</t>
+          <t>E3-TC9</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Risk seviyesine göre filtreleme</t>
+          <t>Rapor silinince iş kalemleri de silinir</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Yüksek riskli proje mevcut</t>
+          <t>Raporda iş kalemi var</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>riskLevel=YUKSEK</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>GET /api/dashboard/summary?riskLevel=YUKSEK</t>
+          <t>DELETE /api/reports/{id}; sonra GET iş kalemi</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Yalnızca yüksek riskli projeler</t>
+          <t>204; iş kalemi 404 (cascade)</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Yalnızca YUKSEK döndü</t>
+          <t>204 + 404</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -1773,21 +1765,29 @@
       <c r="K31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr"/>
-      <c r="B32" s="3" t="inlineStr"/>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>E4</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>CTO Dashboard</t>
+        </is>
+      </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>E4-TC3</t>
+          <t>E4-TC1</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Raporu olmayan proje özeti</t>
+          <t>Portföy özetini görüntüleme</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Raporsuz proje mevcut</t>
+          <t>Kayıtlı projeler</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -1802,12 +1802,12 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Proje listelenir; hasReport=false, ilerleme boş</t>
+          <t>200; tüm projeler + sayaçlar</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>hasReport=false</t>
+          <t>200, özet döndü</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -1822,37 +1822,37 @@
       <c r="B33" s="3" t="inlineStr"/>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>E4-TC4</t>
+          <t>E4-TC2</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Boş portföy (hiç proje yok)</t>
+          <t>Risk seviyesine göre filtreleme</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Veritabanında proje yok</t>
+          <t>Yüksek riskli proje mevcut</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>riskLevel=YUKSEK</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>GET /api/dashboard/summary</t>
+          <t>GET /api/dashboard/summary?riskLevel=YUKSEK</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>totalProjects=0; liste boş; sayaçlar 0</t>
+          <t>Yalnızca yüksek riskli projeler</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>0, boş liste</t>
+          <t>Yalnızca YUKSEK döndü</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -1860,48 +1860,44 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t>Birim testiyle doğrulandı</t>
-        </is>
-      </c>
+      <c r="K33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr"/>
       <c r="B34" s="3" t="inlineStr"/>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>E4-TC5</t>
+          <t>E4-TC3</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Geçersiz risk filtresi</t>
+          <t>Raporu olmayan proje özeti</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Raporsuz proje mevcut</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>riskLevel=COK_YUKSEK</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>GET /api/dashboard/summary?riskLevel=COK_YUKSEK</t>
+          <t>GET /api/dashboard/summary</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>400 INVALID_REQUEST</t>
+          <t>Proje listelenir; hasReport=false, ilerleme boş</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>400 döndü</t>
+          <t>hasReport=false</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -1909,36 +1905,24 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t>H-3 düzeltmesi sonrası</t>
-        </is>
-      </c>
+      <c r="K34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>E5</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Genel / sistem</t>
-        </is>
-      </c>
+      <c r="A35" s="3" t="inlineStr"/>
+      <c r="B35" s="3" t="inlineStr"/>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>E5-TC1</t>
+          <t>E4-TC4</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Sağlık kontrolü</t>
+          <t>Boş portföy (hiç proje yok)</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Uygulama ayakta</t>
+          <t>Veritabanında proje yok</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -1948,17 +1932,17 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>GET /api/health</t>
+          <t>GET /api/dashboard/summary</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>200; status UP, databaseStatus UP</t>
+          <t>totalProjects=0; liste boş; sayaçlar 0</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>200, UP</t>
+          <t>0, boş liste</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -1966,19 +1950,23 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K35" s="3" t="inlineStr"/>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>Birim testiyle doğrulandı</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr"/>
       <c r="B36" s="3" t="inlineStr"/>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>E5-TC2</t>
+          <t>E4-TC5</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Tanımsız endpoint çağırma</t>
+          <t>Geçersiz risk filtresi</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -1988,22 +1976,22 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>riskLevel=COK_YUKSEK</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>GET /api/olmayan-endpoint</t>
+          <t>GET /api/dashboard/summary?riskLevel=COK_YUKSEK</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>404 RESOURCE_NOT_FOUND</t>
+          <t>400 INVALID_REQUEST</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>404 döndü</t>
+          <t>400 döndü</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -2011,24 +1999,36 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K36" s="3" t="inlineStr"/>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>H-3: ilk testte 500 (FAIL) idi; parametre tip doğrulaması eklendikten sonra PASS</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr"/>
-      <c r="B37" s="3" t="inlineStr"/>
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>E5</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Genel / sistem</t>
+        </is>
+      </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>E5-TC3</t>
+          <t>E5-TC1</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Desteklenmeyen HTTP metodu</t>
+          <t>Sağlık kontrolü</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Uygulama ayakta</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -2038,17 +2038,17 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>PATCH /api/health</t>
+          <t>GET /api/health</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>405 METHOD_NOT_ALLOWED</t>
+          <t>200; status UP, databaseStatus UP</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>405 döndü</t>
+          <t>200, UP</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -2063,12 +2063,12 @@
       <c r="B38" s="3" t="inlineStr"/>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>E5-TC4</t>
+          <t>E5-TC2</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Beklenmeyen sunucu hatası</t>
+          <t>Tanımsız endpoint çağırma</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2078,22 +2078,22 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>(sunucu içi beklenmeyen hata)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>İç hata tetiklenir</t>
+          <t>GET /api/olmayan-endpoint</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>500 INTERNAL_ERROR; teknik detay sızmaz, loglanır</t>
+          <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>500, genel mesaj</t>
+          <t>404 döndü</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -2101,56 +2101,146 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr">
-        <is>
-          <t>Hata yönetimi testi</t>
-        </is>
-      </c>
+      <c r="K38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr"/>
       <c r="B39" s="3" t="inlineStr"/>
       <c r="C39" s="3" t="inlineStr">
         <is>
+          <t>E5-TC3</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Desteklenmeyen HTTP metodu</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>PATCH /api/health</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>405 METHOD_NOT_ALLOWED</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>405 döndü</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr"/>
+      <c r="B40" s="3" t="inlineStr"/>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>E5-TC4</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Beklenmeyen sunucu hatası</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>(sunucu içi beklenmeyen hata)</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>İç hata tetiklenir</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>500 INTERNAL_ERROR; teknik detay sızmaz, loglanır</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>500, genel mesaj</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Hata yönetimi testi</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr"/>
+      <c r="B41" s="3" t="inlineStr"/>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
           <t>E5-TC5</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>Uygulamanın ayağa kalkması</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Uygulamayı başlat</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>Spring context sorunsuz yüklenir</t>
         </is>
       </c>
-      <c r="I39" s="3" t="inlineStr">
+      <c r="I41" s="3" t="inlineStr">
         <is>
           <t>Yüklendi</t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K39" s="3" t="inlineStr">
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
         <is>
           <t>Smoke/context testi</t>
         </is>

</xml_diff>

<commit_message>
docs: clean up test data (realistic broken JSON, consistent ids, header spacing)
</commit_message>
<xml_diff>
--- a/docs/Test Senaryolari - CTO Takip Sistemi.xlsx
+++ b/docs/Test Senaryolari - CTO Takip Sistemi.xlsx
@@ -72,9 +72,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -474,7 +477,7 @@
           <t>Project</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Haftalık Proje Durum Raporlama ve CTO Takip Sistemi (Backend)</t>
         </is>
@@ -486,7 +489,7 @@
           <t>Testers</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Gökhan Kara</t>
         </is>
@@ -498,1792 +501,1792 @@
           <t>Test Environments</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Lokal: http://localhost:8080  (Swagger UI: /swagger-ui.html)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Scenario ID</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Test Cases</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Expected result</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>E1-SC1</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Proje oluşturma ve silme (geçerli işlemler)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>E1-SC1-TC-Project-1</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Geçerli veriyle proje oluşturma</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Kayıtlı PM (ownerId=1)</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>{"name":"PEYK","status":"DEVAM_EDIYOR","ownerId":1}</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>POST /api/projects</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>201 Created; proje bilgisi döner</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>201, proje oluştu</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
-      <c r="B7" s="4" t="inlineStr"/>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>E1-SC1-TC-Project-2</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Raporu olmayan projeyi silme</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Raporsuz proje</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>id (raporsuz)</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>DELETE /api/projects/{id}</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>204 No Content; proje silinir</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>204, silindi</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>E1-SC2</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Proje işlemlerinde hata/negatif senaryolar</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>E1-SC2-TC-Project-1</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Zorunlu alanlar eksik proje oluşturma</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>POST /api/projects</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>400 VALIDATION_ERROR + fieldErrors</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>400, alan hataları döndü</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>E1-SC2-TC-Project-2</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Çok uzun proje adı (255 karakter üstü)</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>name = 300 karakter</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>POST /api/projects</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>400 VALIDATION_ERROR</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>H-2: ilk testte 500 (FAIL) idi; @Size doğrulaması eklendikten sonra PASS</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
-      <c r="B10" s="4" t="inlineStr"/>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>E1-SC2-TC-Project-3</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Olmayan sorumlu (owner) ile proje</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>{"name":"X","status":"PLANLANDI","ownerId":999}</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>POST /api/projects</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>404 döndü</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="4" t="inlineStr"/>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>E1-SC2-TC-Project-4</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Olmayan proje detayını getirme</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>id=99999</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>GET /api/projects/99999</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>id=9999</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>GET /api/projects/9999</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>404 döndü</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" s="4" t="inlineStr"/>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>E1-SC2-TC-Project-5</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Raporu olan projeyi silme</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Proje 1'in raporu var</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>id=1</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>DELETE /api/projects/1</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>409 RESOURCE_IN_USE</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>409, 'önce raporları silin'</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>H-1: ilk testte 500 (FAIL) idi; silme öncesi rapor kontrolü eklendikten sonra PASS</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>E2-SC1</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Haftalık rapor - geçerli işlemler</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>E2-SC1-TC-Report-1</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Geçerli haftalık rapor oluşturma</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Kayıtlı proje</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>{"weekNumber":25,"reportDate":"2026-08-03","progressStage":"ANALIZ","overallStatus":"YOLUNDA","riskLevel":"DUSUK"}</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>POST /api/projects/{id}/reports</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>201; progressPercentage kademeden türer (25)</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>201, %25</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
-      <c r="B14" s="4" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr"/>
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>E2-SC1-TC-Report-2</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Geçerli ilerleme (bir kademe ileri)</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Rapor kademesi GELISTIRME</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>progressStage=TEST</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>PUT /api/reports/{id}</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>200; yüzde 75'e güncellenir</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>200, %75</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>E2-SC2</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Haftalık rapor - hata/negatif senaryolar</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>E2-SC2-TC-Report-1</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Olmayan projeye rapor ekleme</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>projectId=9999</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>POST /api/projects/9999/reports</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>404 döndü</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>E2-SC2-TC-Report-2</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Aynı proje+hafta için ikinci rapor (oluşturma)</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Proje 1 hafta 29 mevcut</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>weekNumber=29</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>POST /api/projects/1/reports</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>409 DUPLICATE_RESOURCE</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>409 döndü</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
-      <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr"/>
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>E2-SC2-TC-Report-3</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Güncellemede hafta değiştirip çakışma</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>Aynı projede başka hafta raporu var</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>weekNumber = mevcut başka hafta</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>PUT /api/reports/{id}</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>409 DUPLICATE_RESOURCE</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>409 döndü</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr"/>
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>E2-SC2-TC-Report-4</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>İlerleme kademesinde sıra atlama</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Rapor kademesi ANALIZ</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>progressStage=TAMAMLANDI</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>PUT /api/reports/{id}</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>400 BUSINESS_RULE_VIOLATION</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr"/>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr"/>
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>E2-SC2-TC-Report-5</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>İlerleme kademesini geriye alma</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>Rapor kademesi TEST</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>progressStage=ANALIZ</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>PUT /api/reports/{id}</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>400 BUSINESS_RULE_VIOLATION</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr"/>
-      <c r="B20" s="4" t="inlineStr"/>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>E2-SC2-TC-Report-6</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>Tanımsız enum değeri ile rapor</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>progressStage="COK_ILERI"</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>POST /api/projects/{id}/reports</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>400 INVALID_REQUEST</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr"/>
-      <c r="B21" s="4" t="inlineStr"/>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr"/>
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>E2-SC2-TC-Report-7</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Geçersiz tarih formatı ile rapor</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>reportDate="2026-13-99"</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>POST /api/projects/{id}/reports</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>400 INVALID_REQUEST</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr"/>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr"/>
-      <c r="B22" s="4" t="inlineStr"/>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr"/>
+      <c r="B22" s="5" t="inlineStr"/>
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>E2-SC2-TC-Report-8</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Bozuk JSON gövdesi ile istek</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>{ bozuk</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>{"weekNumber": 25   (kapanış } eksik)</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>POST /api/projects/{id}/reports</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>400 INVALID_REQUEST</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr"/>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>E3-SC1</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>İş kalemi - geçerli işlemler</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>E3-SC1-TC-WorkItem-1</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Geçerli iş kalemi ekleme</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Kayıtlı rapor</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>{"title":"Analiz görüşmesi","status":"DEVAM_EDIYOR","assignee":"Ayşe"}</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>POST /api/reports/{id}/work-items</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>201 Created</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>201, iş kalemi eklendi</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr"/>
-      <c r="B24" s="4" t="inlineStr"/>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr"/>
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>E3-SC1-TC-WorkItem-2</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>İş kalemi güncelleme (başarılı)</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>Kayıtlı iş kalemi</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>{"title":"Güncellendi","status":"TAMAMLANDI"}</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>PUT /api/work-items/{id}</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>200; alanlar güncellenir</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>200, güncellendi</t>
         </is>
       </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr"/>
-      <c r="B25" s="4" t="inlineStr"/>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>E3-SC1-TC-WorkItem-3</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>İş kalemi silme (başarılı)</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>Kayıtlı iş kalemi</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>DELETE /api/work-items/{id}</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>204 No Content</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>204, silindi</t>
         </is>
       </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr"/>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr"/>
+      <c r="B26" s="5" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>E3-SC1-TC-WorkItem-4</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Canlı task sayımı (DEVAM_EDIYOR)</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Raporda 1 DEVAM_EDIYOR iş kalemi</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>GET /api/reports/{id}</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>liveTaskCount = 1</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="I26" s="5" t="inlineStr">
         <is>
           <t>liveTaskCount = 1</t>
         </is>
       </c>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
         <is>
           <t>Ayrı alan tutulmaz, türetilir</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr"/>
-      <c r="B27" s="4" t="inlineStr"/>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr"/>
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>E3-SC1-TC-WorkItem-5</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>Rapor silinince iş kalemleri de silinir</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>Raporda iş kalemi var</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>DELETE /api/reports/{id}; sonra GET iş kalemi</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>204; iş kalemi 404 (cascade)</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>204 + 404</t>
         </is>
       </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>E3-SC2</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>İş kalemi - hata/negatif senaryolar</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>E3-SC2-TC-WorkItem-1</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>Boş başlıkla iş kalemi ekleme</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>{"title":"","status":"PLANLANDI"}</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>POST /api/reports/{id}/work-items</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>400 VALIDATION_ERROR</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I28" s="5" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr"/>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr"/>
-      <c r="B29" s="4" t="inlineStr"/>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr"/>
+      <c r="B29" s="5" t="inlineStr"/>
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>E3-SC2-TC-WorkItem-2</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>Olmayan rapora iş kalemi ekleme</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>reportId=999</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>POST /api/reports/999/work-items</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>reportId=9999</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>POST /api/reports/9999/work-items</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>404 döndü</t>
         </is>
       </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr"/>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr"/>
-      <c r="B30" s="4" t="inlineStr"/>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr"/>
+      <c r="B30" s="5" t="inlineStr"/>
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>E3-SC2-TC-WorkItem-3</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>Olmayan iş kalemini getirme</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>id=9999</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>GET /api/work-items/9999</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I30" s="5" t="inlineStr">
         <is>
           <t>404 döndü</t>
         </is>
       </c>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K30" s="4" t="inlineStr"/>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr"/>
-      <c r="B31" s="4" t="inlineStr"/>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr"/>
+      <c r="B31" s="5" t="inlineStr"/>
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>E3-SC2-TC-WorkItem-4</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>Olmayan iş kalemini silme</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>id=9999</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>DELETE /api/work-items/9999</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>404 döndü</t>
         </is>
       </c>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K31" s="4" t="inlineStr"/>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>E4-SC1</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>CTO Dashboard - geçerli görüntüleme ve filtre</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>E4-SC1-TC-Dashboard-1</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>Portföy özetini görüntüleme</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>Kayıtlı projeler</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>GET /api/dashboard/summary</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>200; tüm projeler + sayaçlar</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I32" s="5" t="inlineStr">
         <is>
           <t>200, özet döndü</t>
         </is>
       </c>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr"/>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr"/>
-      <c r="B33" s="4" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr"/>
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>E4-SC1-TC-Dashboard-2</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>Risk seviyesine göre filtreleme</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>Yüksek riskli proje mevcut</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>riskLevel=YUKSEK</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>GET /api/dashboard/summary?riskLevel=YUKSEK</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>Yalnızca yüksek riskli projeler</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="I33" s="5" t="inlineStr">
         <is>
           <t>Yalnızca YUKSEK döndü</t>
         </is>
       </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K33" s="4" t="inlineStr"/>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr"/>
-      <c r="B34" s="4" t="inlineStr"/>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>E4-SC1-TC-Dashboard-3</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>Raporu olmayan proje özeti</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>Raporsuz proje mevcut</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>GET /api/dashboard/summary</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>Proje listelenir; hasReport=false, ilerleme boş</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I34" s="5" t="inlineStr">
         <is>
           <t>hasReport=false</t>
         </is>
       </c>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K34" s="4" t="inlineStr"/>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr"/>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="A35" s="5" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>E4-SC1-TC-Dashboard-4</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>Boş portföy (hiç proje yok)</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>Veritabanında proje yok</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>GET /api/dashboard/summary</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="H35" s="5" t="inlineStr">
         <is>
           <t>totalProjects=0; liste boş; sayaçlar 0</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="I35" s="5" t="inlineStr">
         <is>
           <t>0, boş liste</t>
         </is>
       </c>
-      <c r="J35" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
         <is>
           <t>Birim testiyle doğrulandı</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>E4-SC2</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>CTO Dashboard - hata/negatif senaryolar</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>E4-SC2-TC-Dashboard-1</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>Geçersiz risk filtresi</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>riskLevel=COK_YUKSEK</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>GET /api/dashboard/summary?riskLevel=COK_YUKSEK</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>400 INVALID_REQUEST</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="I36" s="5" t="inlineStr">
         <is>
           <t>400 döndü</t>
         </is>
       </c>
-      <c r="J36" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K36" s="4" t="inlineStr">
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
         <is>
           <t>H-3: ilk testte 500 (FAIL) idi; parametre tip doğrulaması eklendikten sonra PASS</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>E5-SC1</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>Genel / sistem - geçerli</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>E5-SC1-TC-System-1</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>Sağlık kontrolü</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>Uygulama ayakta</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>GET /api/health</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>200; status UP, databaseStatus UP</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr">
+      <c r="I37" s="5" t="inlineStr">
         <is>
           <t>200, UP</t>
         </is>
       </c>
-      <c r="J37" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K37" s="4" t="inlineStr"/>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr"/>
-      <c r="B38" s="4" t="inlineStr"/>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="A38" s="5" t="inlineStr"/>
+      <c r="B38" s="5" t="inlineStr"/>
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>E5-SC1-TC-System-2</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>Uygulamanın ayağa kalkması</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>Uygulamayı başlat</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>Spring context sorunsuz yüklenir</t>
         </is>
       </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="I38" s="5" t="inlineStr">
         <is>
           <t>Yüklendi</t>
         </is>
       </c>
-      <c r="J38" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr">
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
         <is>
           <t>Smoke/context testi</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>E5-SC2</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Genel / sistem - hata/negatif</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>E5-SC2-TC-System-1</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>Tanımsız endpoint çağırma</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>GET /api/olmayan-endpoint</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>404 RESOURCE_NOT_FOUND</t>
         </is>
       </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="I39" s="5" t="inlineStr">
         <is>
           <t>404 döndü</t>
         </is>
       </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr"/>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr"/>
-      <c r="B40" s="4" t="inlineStr"/>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="A40" s="5" t="inlineStr"/>
+      <c r="B40" s="5" t="inlineStr"/>
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>E5-SC2-TC-System-2</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>Desteklenmeyen HTTP metodu</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>PATCH /api/health</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>405 METHOD_NOT_ALLOWED</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr">
+      <c r="I40" s="5" t="inlineStr">
         <is>
           <t>405 döndü</t>
         </is>
       </c>
-      <c r="J40" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr"/>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr"/>
-      <c r="B41" s="4" t="inlineStr"/>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr"/>
+      <c r="B41" s="5" t="inlineStr"/>
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>E5-SC2-TC-System-3</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>Beklenmeyen sunucu hatası</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>(sunucu içi beklenmeyen hata)</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>İç hata tetiklenir</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Beklenmeyen çalışma zamanı hatası oluşur (otomatik testle simüle edilir)</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
         <is>
           <t>500 INTERNAL_ERROR; teknik detay sızmaz, loglanır</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="I41" s="5" t="inlineStr">
         <is>
           <t>500, genel mesaj</t>
         </is>
       </c>
-      <c r="J41" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr">
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
         <is>
           <t>Hata yönetimi testi</t>
         </is>

</xml_diff>

<commit_message>
docs: fill test data for id-based operations in test scenarios
</commit_message>
<xml_diff>
--- a/docs/Test Senaryolari - CTO Takip Sistemi.xlsx
+++ b/docs/Test Senaryolari - CTO Takip Sistemi.xlsx
@@ -637,7 +637,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>id = raporsuz bir projenin id'si</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>id = mevcut iş kaleminin id'si</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>id = mevcut raporun id'si</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>id = mevcut raporun id'si</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">

</xml_diff>